<commit_message>
Fixed two carmine red values from NA to 300 min, the upper limit accordign to Ana
</commit_message>
<xml_diff>
--- a/Data/motor_performance/data_clean_ga.xlsx
+++ b/Data/motor_performance/data_clean_ga.xlsx
@@ -5,18 +5,18 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/giacomo/Documents/git_repos/MazmanianS_MoiseyenkoA/Data/motor_performance/clean_ga/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/giacomo/Documents/git_repos/MazmanianS_MoiseyenkoA/Data/motor_performance/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9C669F59-5302-F945-AA51-0CFAA3E7DD91}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83D1E0F1-C150-8D46-885A-B6CFB407CC08}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="25700" yWindow="660" windowWidth="25360" windowHeight="27980" activeTab="1" xr2:uid="{386C456C-A0E0-4242-B482-FC80BD37ADC9}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17520" xr2:uid="{386C456C-A0E0-4242-B482-FC80BD37ADC9}"/>
   </bookViews>
   <sheets>
     <sheet name="motor_tests_together_clean" sheetId="1" r:id="rId1"/>
     <sheet name="motor_tests_with_metagenome" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -146,18 +146,12 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -172,17 +166,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="2" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="20" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -583,7 +574,7 @@
       <c r="R1" t="s">
         <v>22</v>
       </c>
-      <c r="V1" s="6"/>
+      <c r="V1" s="5"/>
     </row>
     <row r="2" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A2">
@@ -640,7 +631,7 @@
       <c r="R2" s="1">
         <v>10</v>
       </c>
-      <c r="V2" s="6"/>
+      <c r="V2" s="5"/>
     </row>
     <row r="3" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A3">
@@ -697,7 +688,7 @@
       <c r="R3" s="1">
         <v>0</v>
       </c>
-      <c r="V3" s="6"/>
+      <c r="V3" s="5"/>
     </row>
     <row r="4" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A4">
@@ -754,7 +745,7 @@
       <c r="R4" s="1">
         <v>1</v>
       </c>
-      <c r="V4" s="6"/>
+      <c r="V4" s="5"/>
     </row>
     <row r="5" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A5">
@@ -811,7 +802,7 @@
       <c r="R5" s="1">
         <v>6</v>
       </c>
-      <c r="V5" s="6"/>
+      <c r="V5" s="5"/>
     </row>
     <row r="6" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A6">
@@ -868,7 +859,7 @@
       <c r="R6" s="1">
         <v>2</v>
       </c>
-      <c r="V6" s="6"/>
+      <c r="V6" s="5"/>
     </row>
     <row r="7" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A7">
@@ -925,7 +916,7 @@
       <c r="R7" s="1">
         <v>10</v>
       </c>
-      <c r="V7" s="6"/>
+      <c r="V7" s="5"/>
     </row>
     <row r="8" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A8">
@@ -982,7 +973,7 @@
       <c r="R8" s="1">
         <v>16</v>
       </c>
-      <c r="V8" s="6"/>
+      <c r="V8" s="5"/>
     </row>
     <row r="9" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A9">
@@ -1039,7 +1030,7 @@
       <c r="R9" s="1">
         <v>34</v>
       </c>
-      <c r="V9" s="6"/>
+      <c r="V9" s="5"/>
     </row>
     <row r="10" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A10">
@@ -1096,7 +1087,7 @@
       <c r="R10" s="1">
         <v>43</v>
       </c>
-      <c r="V10" s="6"/>
+      <c r="V10" s="5"/>
     </row>
     <row r="11" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A11">
@@ -1153,7 +1144,7 @@
       <c r="R11" s="1">
         <v>19</v>
       </c>
-      <c r="V11" s="6"/>
+      <c r="V11" s="5"/>
     </row>
     <row r="12" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A12">
@@ -1210,7 +1201,7 @@
       <c r="R12" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="V12" s="6"/>
+      <c r="V12" s="5"/>
     </row>
     <row r="13" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A13">
@@ -1267,7 +1258,7 @@
       <c r="R13" s="1">
         <v>26</v>
       </c>
-      <c r="V13" s="6"/>
+      <c r="V13" s="5"/>
     </row>
     <row r="14" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A14">
@@ -1324,7 +1315,7 @@
       <c r="R14" s="1">
         <v>29</v>
       </c>
-      <c r="V14" s="6"/>
+      <c r="V14" s="5"/>
     </row>
     <row r="15" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A15">
@@ -1381,7 +1372,7 @@
       <c r="R15" s="1">
         <v>21</v>
       </c>
-      <c r="V15" s="6"/>
+      <c r="V15" s="5"/>
     </row>
     <row r="16" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A16">
@@ -1438,7 +1429,7 @@
       <c r="R16" s="1">
         <v>38</v>
       </c>
-      <c r="V16" s="6"/>
+      <c r="V16" s="5"/>
     </row>
     <row r="17" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A17">
@@ -1495,7 +1486,7 @@
       <c r="R17" s="1">
         <v>0</v>
       </c>
-      <c r="V17" s="6"/>
+      <c r="V17" s="5"/>
     </row>
     <row r="18" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A18">
@@ -1552,7 +1543,7 @@
       <c r="R18" s="1">
         <v>25</v>
       </c>
-      <c r="V18" s="6"/>
+      <c r="V18" s="5"/>
     </row>
     <row r="19" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A19">
@@ -1609,7 +1600,7 @@
       <c r="R19" s="1">
         <v>32</v>
       </c>
-      <c r="V19" s="6"/>
+      <c r="V19" s="5"/>
     </row>
     <row r="20" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A20">
@@ -1666,7 +1657,7 @@
       <c r="R20" s="1">
         <v>8</v>
       </c>
-      <c r="V20" s="6"/>
+      <c r="V20" s="5"/>
     </row>
     <row r="21" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A21">
@@ -1723,7 +1714,7 @@
       <c r="R21" s="1">
         <v>12</v>
       </c>
-      <c r="V21" s="6"/>
+      <c r="V21" s="5"/>
     </row>
     <row r="22" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A22">
@@ -1780,7 +1771,7 @@
       <c r="R22" s="1">
         <v>29</v>
       </c>
-      <c r="V22" s="6"/>
+      <c r="V22" s="5"/>
     </row>
     <row r="23" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A23">
@@ -1837,7 +1828,7 @@
       <c r="R23" s="3">
         <v>7.78</v>
       </c>
-      <c r="V23" s="6"/>
+      <c r="V23" s="5"/>
     </row>
     <row r="24" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A24">
@@ -1894,7 +1885,7 @@
       <c r="R24" s="3">
         <v>4.8600000000000003</v>
       </c>
-      <c r="V24" s="6"/>
+      <c r="V24" s="5"/>
     </row>
     <row r="25" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A25">
@@ -1951,7 +1942,7 @@
       <c r="R25" s="3">
         <v>4.8600000000000003</v>
       </c>
-      <c r="V25" s="6"/>
+      <c r="V25" s="5"/>
     </row>
     <row r="26" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A26">
@@ -2008,7 +1999,7 @@
       <c r="R26" s="3">
         <v>0</v>
       </c>
-      <c r="V26" s="6"/>
+      <c r="V26" s="5"/>
     </row>
     <row r="27" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A27">
@@ -2065,7 +2056,7 @@
       <c r="R27" s="3">
         <v>8.75</v>
       </c>
-      <c r="V27" s="6"/>
+      <c r="V27" s="5"/>
     </row>
     <row r="28" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A28">
@@ -2122,7 +2113,7 @@
       <c r="R28" s="3">
         <v>3.89</v>
       </c>
-      <c r="V28" s="6"/>
+      <c r="V28" s="5"/>
     </row>
     <row r="29" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A29">
@@ -2179,7 +2170,7 @@
       <c r="R29" s="3">
         <v>18.47</v>
       </c>
-      <c r="V29" s="6"/>
+      <c r="V29" s="5"/>
     </row>
     <row r="30" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A30">
@@ -2236,7 +2227,7 @@
       <c r="R30" s="3">
         <v>0</v>
       </c>
-      <c r="V30" s="6"/>
+      <c r="V30" s="5"/>
     </row>
     <row r="31" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A31">
@@ -2293,7 +2284,7 @@
       <c r="R31" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="V31" s="6"/>
+      <c r="V31" s="5"/>
     </row>
     <row r="32" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A32">
@@ -2350,7 +2341,7 @@
       <c r="R32" s="3">
         <v>20.420000000000002</v>
       </c>
-      <c r="V32" s="6"/>
+      <c r="V32" s="5"/>
     </row>
     <row r="33" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A33">
@@ -2401,13 +2392,13 @@
       <c r="P33" s="1">
         <v>47.058823500000003</v>
       </c>
-      <c r="Q33" s="5">
-        <v>0</v>
+      <c r="Q33" s="6">
+        <v>300</v>
       </c>
       <c r="R33" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="V33" s="6"/>
+      <c r="V33" s="5"/>
     </row>
     <row r="34" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A34">
@@ -2458,13 +2449,13 @@
       <c r="P34" s="1">
         <v>33.3333333</v>
       </c>
-      <c r="Q34" s="5">
-        <v>0</v>
+      <c r="Q34" s="6">
+        <v>300</v>
       </c>
       <c r="R34" s="3">
         <v>26.25</v>
       </c>
-      <c r="V34" s="6"/>
+      <c r="V34" s="5"/>
     </row>
     <row r="35" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A35">
@@ -2521,7 +2512,7 @@
       <c r="R35" s="3">
         <v>23.33</v>
       </c>
-      <c r="V35" s="6"/>
+      <c r="V35" s="5"/>
     </row>
     <row r="36" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A36">
@@ -2578,7 +2569,7 @@
       <c r="R36" s="3">
         <v>35</v>
       </c>
-      <c r="V36" s="6"/>
+      <c r="V36" s="5"/>
     </row>
     <row r="37" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A37">
@@ -2635,7 +2626,7 @@
       <c r="R37" s="3">
         <v>0.97</v>
       </c>
-      <c r="V37" s="6"/>
+      <c r="V37" s="5"/>
     </row>
     <row r="38" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A38">
@@ -2692,7 +2683,7 @@
       <c r="R38" s="3">
         <v>16.53</v>
       </c>
-      <c r="V38" s="6"/>
+      <c r="V38" s="5"/>
     </row>
     <row r="39" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A39">
@@ -2749,7 +2740,7 @@
       <c r="R39" s="3">
         <v>0</v>
       </c>
-      <c r="V39" s="6"/>
+      <c r="V39" s="5"/>
     </row>
     <row r="40" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A40">
@@ -2806,64 +2797,64 @@
       <c r="R40" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="V40" s="6"/>
+      <c r="V40" s="5"/>
     </row>
     <row r="41" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A41" s="7">
-        <v>2</v>
-      </c>
-      <c r="B41" s="8" t="s">
-        <v>7</v>
-      </c>
-      <c r="C41" s="7" t="s">
+      <c r="A41">
+        <v>2</v>
+      </c>
+      <c r="B41" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C41" t="s">
         <v>8</v>
       </c>
-      <c r="D41" s="7">
+      <c r="D41">
         <v>15</v>
       </c>
-      <c r="E41" s="8">
+      <c r="E41" s="1">
         <v>2362</v>
       </c>
-      <c r="F41" s="7">
+      <c r="F41">
         <v>4.4550000000000001</v>
       </c>
-      <c r="G41" s="7">
+      <c r="G41">
         <v>11</v>
       </c>
-      <c r="H41" s="8">
+      <c r="H41" s="1">
         <v>9</v>
       </c>
-      <c r="I41" s="8">
+      <c r="I41" s="1">
         <v>3.55</v>
       </c>
-      <c r="J41" s="8" t="s">
+      <c r="J41" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K41" s="8">
+      <c r="K41" s="1">
         <v>1.73</v>
       </c>
-      <c r="L41" s="8">
+      <c r="L41" s="1">
         <v>0</v>
       </c>
-      <c r="M41" s="8">
+      <c r="M41" s="1">
         <v>4</v>
       </c>
-      <c r="N41" s="8">
+      <c r="N41" s="1">
         <v>4</v>
       </c>
-      <c r="O41" s="8">
+      <c r="O41" s="1">
         <v>3</v>
       </c>
-      <c r="P41" s="8">
+      <c r="P41" s="1">
         <v>53.424657500000002</v>
       </c>
-      <c r="Q41" s="8">
+      <c r="Q41" s="1">
         <v>203.99999999999991</v>
       </c>
-      <c r="R41" s="9">
+      <c r="R41" s="3">
         <v>8.75</v>
       </c>
-      <c r="V41" s="6"/>
+      <c r="V41" s="5"/>
     </row>
     <row r="42" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A42">
@@ -2920,7 +2911,7 @@
       <c r="R42" t="s">
         <v>9</v>
       </c>
-      <c r="V42" s="6"/>
+      <c r="V42" s="5"/>
     </row>
     <row r="43" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A43">
@@ -2977,7 +2968,7 @@
       <c r="R43">
         <v>27.000000000000064</v>
       </c>
-      <c r="V43" s="6"/>
+      <c r="V43" s="5"/>
     </row>
     <row r="44" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A44">
@@ -3034,7 +3025,7 @@
       <c r="R44">
         <v>0.99999999999999645</v>
       </c>
-      <c r="V44" s="6"/>
+      <c r="V44" s="5"/>
     </row>
     <row r="45" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A45">
@@ -3091,7 +3082,7 @@
       <c r="R45">
         <v>0</v>
       </c>
-      <c r="V45" s="6"/>
+      <c r="V45" s="5"/>
     </row>
     <row r="46" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A46">
@@ -3148,7 +3139,7 @@
       <c r="R46">
         <v>11.000000000000121</v>
       </c>
-      <c r="V46" s="6"/>
+      <c r="V46" s="5"/>
     </row>
     <row r="47" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A47">
@@ -3205,7 +3196,7 @@
       <c r="R47">
         <v>5.9999999999999787</v>
       </c>
-      <c r="V47" s="6"/>
+      <c r="V47" s="5"/>
     </row>
     <row r="48" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A48">
@@ -3262,7 +3253,7 @@
       <c r="R48">
         <v>0.99999999999999645</v>
       </c>
-      <c r="V48" s="6"/>
+      <c r="V48" s="5"/>
     </row>
     <row r="49" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A49">
@@ -3319,7 +3310,7 @@
       <c r="R49">
         <v>12.999999999999954</v>
       </c>
-      <c r="V49" s="6"/>
+      <c r="V49" s="5"/>
     </row>
     <row r="50" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A50">
@@ -5400,7 +5391,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8EAB2797-AFE9-8F47-86F8-EE6E32CD156D}">
-  <dimension ref="A1:S93"/>
+  <dimension ref="A1:R93"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="14" max="14" width="22.1640625" bestFit="1" customWidth="1"/>
@@ -7563,7 +7554,7 @@
       </c>
     </row>
     <row r="50" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A50" s="6"/>
+      <c r="A50" s="5"/>
     </row>
     <row r="54" spans="1:18" x14ac:dyDescent="0.2">
       <c r="B54" s="1"/>
@@ -7969,7 +7960,7 @@
       <c r="Q80" s="1"/>
       <c r="R80" s="3"/>
     </row>
-    <row r="81" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="81" spans="2:18" x14ac:dyDescent="0.2">
       <c r="B81" s="1"/>
       <c r="E81" s="1"/>
       <c r="H81" s="1"/>
@@ -7984,7 +7975,7 @@
       <c r="Q81" s="1"/>
       <c r="R81" s="3"/>
     </row>
-    <row r="82" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="82" spans="2:18" x14ac:dyDescent="0.2">
       <c r="B82" s="1"/>
       <c r="E82" s="1"/>
       <c r="H82" s="1"/>
@@ -7995,12 +7986,11 @@
       <c r="M82" s="1"/>
       <c r="N82" s="1"/>
       <c r="O82" s="1"/>
-      <c r="P82" s="8"/>
-      <c r="Q82" s="8"/>
-      <c r="R82" s="9"/>
-      <c r="S82" s="7"/>
-    </row>
-    <row r="83" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="P82" s="1"/>
+      <c r="Q82" s="1"/>
+      <c r="R82" s="3"/>
+    </row>
+    <row r="83" spans="2:18" x14ac:dyDescent="0.2">
       <c r="B83" s="1"/>
       <c r="E83" s="1"/>
       <c r="H83" s="1"/>
@@ -8011,12 +8001,11 @@
       <c r="M83" s="1"/>
       <c r="N83" s="1"/>
       <c r="O83" s="1"/>
-      <c r="P83" s="8"/>
-      <c r="Q83" s="8"/>
-      <c r="R83" s="9"/>
-      <c r="S83" s="7"/>
-    </row>
-    <row r="84" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="P83" s="1"/>
+      <c r="Q83" s="1"/>
+      <c r="R83" s="3"/>
+    </row>
+    <row r="84" spans="2:18" x14ac:dyDescent="0.2">
       <c r="B84" s="1"/>
       <c r="E84" s="1"/>
       <c r="H84" s="1"/>
@@ -8027,12 +8016,11 @@
       <c r="M84" s="1"/>
       <c r="N84" s="1"/>
       <c r="O84" s="1"/>
-      <c r="P84" s="8"/>
-      <c r="Q84" s="8"/>
-      <c r="R84" s="9"/>
-      <c r="S84" s="7"/>
-    </row>
-    <row r="85" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="P84" s="1"/>
+      <c r="Q84" s="1"/>
+      <c r="R84" s="3"/>
+    </row>
+    <row r="85" spans="2:18" x14ac:dyDescent="0.2">
       <c r="B85" s="1"/>
       <c r="E85" s="1"/>
       <c r="H85" s="1"/>
@@ -8043,12 +8031,11 @@
       <c r="M85" s="2"/>
       <c r="N85" s="2"/>
       <c r="O85" s="2"/>
-      <c r="P85" s="8"/>
-      <c r="Q85" s="8"/>
-      <c r="R85" s="9"/>
-      <c r="S85" s="7"/>
-    </row>
-    <row r="86" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="P85" s="1"/>
+      <c r="Q85" s="1"/>
+      <c r="R85" s="3"/>
+    </row>
+    <row r="86" spans="2:18" x14ac:dyDescent="0.2">
       <c r="B86" s="1"/>
       <c r="E86" s="1"/>
       <c r="H86" s="1"/>
@@ -8059,12 +8046,11 @@
       <c r="M86" s="1"/>
       <c r="N86" s="1"/>
       <c r="O86" s="1"/>
-      <c r="P86" s="8"/>
-      <c r="Q86" s="8"/>
-      <c r="R86" s="9"/>
-      <c r="S86" s="7"/>
-    </row>
-    <row r="87" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="P86" s="1"/>
+      <c r="Q86" s="1"/>
+      <c r="R86" s="3"/>
+    </row>
+    <row r="87" spans="2:18" x14ac:dyDescent="0.2">
       <c r="B87" s="1"/>
       <c r="E87" s="1"/>
       <c r="H87" s="1"/>
@@ -8075,12 +8061,11 @@
       <c r="M87" s="1"/>
       <c r="N87" s="1"/>
       <c r="O87" s="1"/>
-      <c r="P87" s="8"/>
-      <c r="Q87" s="8"/>
-      <c r="R87" s="9"/>
-      <c r="S87" s="7"/>
-    </row>
-    <row r="88" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="P87" s="1"/>
+      <c r="Q87" s="1"/>
+      <c r="R87" s="3"/>
+    </row>
+    <row r="88" spans="2:18" x14ac:dyDescent="0.2">
       <c r="B88" s="1"/>
       <c r="E88" s="1"/>
       <c r="H88" s="1"/>
@@ -8091,12 +8076,11 @@
       <c r="M88" s="1"/>
       <c r="N88" s="1"/>
       <c r="O88" s="1"/>
-      <c r="P88" s="8"/>
-      <c r="Q88" s="8"/>
-      <c r="R88" s="9"/>
-      <c r="S88" s="7"/>
-    </row>
-    <row r="89" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="P88" s="1"/>
+      <c r="Q88" s="1"/>
+      <c r="R88" s="3"/>
+    </row>
+    <row r="89" spans="2:18" x14ac:dyDescent="0.2">
       <c r="B89" s="1"/>
       <c r="E89" s="1"/>
       <c r="H89" s="1"/>
@@ -8107,12 +8091,11 @@
       <c r="M89" s="1"/>
       <c r="N89" s="1"/>
       <c r="O89" s="1"/>
-      <c r="P89" s="8"/>
-      <c r="Q89" s="8"/>
-      <c r="R89" s="9"/>
-      <c r="S89" s="7"/>
-    </row>
-    <row r="90" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="P89" s="1"/>
+      <c r="Q89" s="1"/>
+      <c r="R89" s="3"/>
+    </row>
+    <row r="90" spans="2:18" x14ac:dyDescent="0.2">
       <c r="B90" s="1"/>
       <c r="E90" s="1"/>
       <c r="H90" s="1"/>
@@ -8127,7 +8110,7 @@
       <c r="Q90" s="1"/>
       <c r="R90" s="3"/>
     </row>
-    <row r="91" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="91" spans="2:18" x14ac:dyDescent="0.2">
       <c r="B91" s="1"/>
       <c r="E91" s="1"/>
       <c r="H91" s="1"/>
@@ -8142,7 +8125,7 @@
       <c r="Q91" s="1"/>
       <c r="R91" s="3"/>
     </row>
-    <row r="92" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="92" spans="2:18" x14ac:dyDescent="0.2">
       <c r="B92" s="1"/>
       <c r="E92" s="1"/>
       <c r="H92" s="1"/>
@@ -8157,25 +8140,20 @@
       <c r="Q92" s="1"/>
       <c r="R92" s="4"/>
     </row>
-    <row r="93" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A93" s="7"/>
-      <c r="B93" s="8"/>
-      <c r="C93" s="7"/>
-      <c r="D93" s="7"/>
-      <c r="E93" s="8"/>
-      <c r="F93" s="7"/>
-      <c r="G93" s="7"/>
-      <c r="H93" s="8"/>
-      <c r="I93" s="8"/>
-      <c r="J93" s="8"/>
-      <c r="K93" s="8"/>
-      <c r="L93" s="8"/>
-      <c r="M93" s="8"/>
-      <c r="N93" s="8"/>
-      <c r="O93" s="8"/>
-      <c r="P93" s="8"/>
-      <c r="Q93" s="8"/>
-      <c r="R93" s="9"/>
+    <row r="93" spans="2:18" x14ac:dyDescent="0.2">
+      <c r="B93" s="1"/>
+      <c r="E93" s="1"/>
+      <c r="H93" s="1"/>
+      <c r="I93" s="1"/>
+      <c r="J93" s="1"/>
+      <c r="K93" s="1"/>
+      <c r="L93" s="1"/>
+      <c r="M93" s="1"/>
+      <c r="N93" s="1"/>
+      <c r="O93" s="1"/>
+      <c r="P93" s="1"/>
+      <c r="Q93" s="1"/>
+      <c r="R93" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
mice 2374 2377 carmine red time set to 480 min
</commit_message>
<xml_diff>
--- a/Data/motor_performance/data_clean_ga.xlsx
+++ b/Data/motor_performance/data_clean_ga.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/giacomo/Documents/git_repos/MazmanianS_MoiseyenkoA/Data/motor_performance/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83D1E0F1-C150-8D46-885A-B6CFB407CC08}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{476DB2C5-3E79-924A-9C71-30D1BE72F5FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17520" xr2:uid="{386C456C-A0E0-4242-B482-FC80BD37ADC9}"/>
   </bookViews>
@@ -166,14 +166,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="2" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="20" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2392,8 +2391,8 @@
       <c r="P33" s="1">
         <v>47.058823500000003</v>
       </c>
-      <c r="Q33" s="6">
-        <v>300</v>
+      <c r="Q33" s="1">
+        <v>480</v>
       </c>
       <c r="R33" s="3" t="s">
         <v>9</v>
@@ -2449,8 +2448,8 @@
       <c r="P34" s="1">
         <v>33.3333333</v>
       </c>
-      <c r="Q34" s="6">
-        <v>300</v>
+      <c r="Q34" s="1">
+        <v>480</v>
       </c>
       <c r="R34" s="3">
         <v>26.25</v>

</xml_diff>

<commit_message>
Renamed sheets of excel file
</commit_message>
<xml_diff>
--- a/Data/motor_performance/data_clean_ga.xlsx
+++ b/Data/motor_performance/data_clean_ga.xlsx
@@ -8,13 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/giacomo/Documents/git_repos/MazmanianS_MoiseyenkoA/Data/motor_performance/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{476DB2C5-3E79-924A-9C71-30D1BE72F5FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F478B5D-8D1E-A943-903A-9B2E31B39786}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17520" xr2:uid="{386C456C-A0E0-4242-B482-FC80BD37ADC9}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17520" activeTab="1" xr2:uid="{386C456C-A0E0-4242-B482-FC80BD37ADC9}"/>
   </bookViews>
   <sheets>
-    <sheet name="motor_tests_together_clean" sheetId="1" r:id="rId1"/>
-    <sheet name="motor_tests_with_metagenome" sheetId="2" r:id="rId2"/>
+    <sheet name="motorTests_2cohorts_clean" sheetId="1" r:id="rId1"/>
+    <sheet name="motorTests_with_metag_data" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>

</xml_diff>